<commit_message>
Dashboard update 2026-08-09 21:25
</commit_message>
<xml_diff>
--- a/excel/Income.xlsx
+++ b/excel/Income.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\Income\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\Income\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D4FFF34-BE26-4879-B255-BD206DF25CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C7F8C6-BDEB-48FD-ADB9-044D09BEE2F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -459,12 +459,6 @@
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -472,6 +466,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1150,22 +1150,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="41" t="s">
+      <c r="A1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="43"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="41"/>
       <c r="M1" s="44" t="s">
         <v>24</v>
       </c>
@@ -1181,12 +1181,12 @@
         <v>24</v>
       </c>
       <c r="V1" s="47"/>
-      <c r="W1" s="41" t="s">
+      <c r="W1" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="X1" s="42"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="43"/>
+      <c r="X1" s="40"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="41"/>
       <c r="AA1" s="4" t="s">
         <v>26</v>
       </c>
@@ -1372,9 +1372,9 @@
         <f>(W3-Q3)/Q3</f>
         <v>1.6666666666666904E-3</v>
       </c>
-      <c r="Z3" s="38" t="e">
+      <c r="Z3" s="38">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>#NUM!</v>
+        <v>2.801214158535004E-2</v>
       </c>
       <c r="AA3" s="36">
         <f>SUM(O3:O100)</f>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="K4" s="19">
         <f ca="1">'19883321'!B12</f>
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="L4" s="19" t="str">
         <f ca="1">'19883321'!P3</f>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="K5" s="19">
         <f ca="1">'20305579'!B12</f>
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="L5" s="19" t="str">
         <f ca="1">'20305579'!P3</f>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="K6" s="19">
         <f ca="1">'20439014'!B12</f>
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="L6" s="19" t="str">
         <f ca="1">'20439014'!P3</f>
@@ -2122,224 +2122,320 @@
       <c r="D3" s="3">
         <v>0</v>
       </c>
-      <c r="K3" s="2"/>
+      <c r="K3" s="3">
+        <f>B3*-1</f>
+        <v>-10</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="3">
+        <f t="shared" ref="K4:K34" si="0">B4*-1</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-      <c r="K9" s="2"/>
+      <c r="K9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
-      <c r="K10" s="2"/>
+      <c r="K10" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
-      <c r="K11" s="2"/>
+      <c r="K11" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="K12" s="2"/>
+      <c r="K12" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="K13" s="2"/>
+      <c r="K13" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-      <c r="K14" s="2"/>
+      <c r="K14" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="K15" s="2"/>
+      <c r="K15" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
-      <c r="K16" s="2"/>
+      <c r="K16" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
-      <c r="K17" s="2"/>
+      <c r="K17" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
-      <c r="K18" s="2"/>
+      <c r="K18" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
-      <c r="K19" s="2"/>
+      <c r="K19" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="15"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
-      <c r="K20" s="2"/>
+      <c r="K20" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
-      <c r="K21" s="2"/>
+      <c r="K21" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
-      <c r="K22" s="2"/>
+      <c r="K22" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
-      <c r="K23" s="2"/>
+      <c r="K23" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
-      <c r="K24" s="2"/>
+      <c r="K24" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="15"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
-      <c r="K25" s="2"/>
+      <c r="K25" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="15"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="K26" s="2"/>
+      <c r="K26" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="15"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
-      <c r="K27" s="2"/>
+      <c r="K27" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
-      <c r="K28" s="2"/>
+      <c r="K28" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
-      <c r="K29" s="2"/>
+      <c r="K29" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
-      <c r="K30" s="2"/>
+      <c r="K30" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="15"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
-      <c r="K31" s="2"/>
+      <c r="K31" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="15"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
-      <c r="K32" s="2"/>
+      <c r="K32" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="15"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
-      <c r="K33" s="2"/>
+      <c r="K33" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="15"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
-      <c r="K34" s="2"/>
+      <c r="K34" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="15"/>
@@ -3499,7 +3595,7 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f ca="1">TODAY()</f>
-        <v>46230</v>
+        <v>46243</v>
       </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -3541,29 +3637,29 @@
       <c r="B1" s="2">
         <v>20439014</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="42"/>
-      <c r="I1" s="43"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="40"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="43"/>
-      <c r="X1" s="41"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="43"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="41"/>
+      <c r="X1" s="39"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="41"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -3886,7 +3982,7 @@
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -4765,20 +4861,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="13" priority="3">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="12" priority="4">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4815,29 +4911,29 @@
       <c r="B1" s="2">
         <v>20305579</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="42"/>
-      <c r="I1" s="43"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="40"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="43"/>
-      <c r="X1" s="41"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="43"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="41"/>
+      <c r="X1" s="39"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="41"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -5160,7 +5256,7 @@
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -6039,20 +6135,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="13" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="12" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6089,29 +6185,29 @@
       <c r="B1" s="2">
         <v>19883321</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="42"/>
-      <c r="I1" s="43"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="40"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="43"/>
-      <c r="X1" s="41"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="43"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="41"/>
+      <c r="X1" s="39"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="41"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -6444,7 +6540,7 @@
       </c>
       <c r="B12" s="19">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="6"/>
@@ -7324,20 +7420,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="7" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="6" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7374,29 +7470,29 @@
       <c r="B1" s="2">
         <v>20191904</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="42"/>
-      <c r="I1" s="43"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="40"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="16"/>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="43"/>
-      <c r="X1" s="41"/>
-      <c r="Y1" s="42"/>
-      <c r="Z1" s="43"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="41"/>
+      <c r="X1" s="39"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="41"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -8606,20 +8702,20 @@
     <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$Z$3="+"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$B$16=$K$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z3">
-    <cfRule type="expression" dxfId="4" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>$Z$3="+"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>